<commit_message>
Data Validator with the all tables were added. The function to check whether it is Table and List is missing.
</commit_message>
<xml_diff>
--- a/IEF_Home/UploadedFiles/1_F_Inputoutput_TABLE_Sample_Test.xlsx
+++ b/IEF_Home/UploadedFiles/1_F_Inputoutput_TABLE_Sample_Test.xlsx
@@ -1,9 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20414"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20415"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{137DAC03-7108-408C-BCAB-4C3DE832CE98}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A2DD7EF-799F-4810-9470-837AE99DF4D2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="9330" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1477" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1477" uniqueCount="258">
   <si>
     <t>Format_Version</t>
   </si>
@@ -789,6 +789,9 @@
   </si>
   <si>
     <t>none1</t>
+  </si>
+  <si>
+    <t>layer1</t>
   </si>
 </sst>
 </file>
@@ -1278,6 +1281,21 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1304,21 +1322,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1677,20 +1680,20 @@
       <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="88" t="s">
+      <c r="B2" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="89"/>
-      <c r="D2" s="90"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="95"/>
       <c r="E2" s="66"/>
-      <c r="F2" s="88" t="s">
+      <c r="F2" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="89"/>
-      <c r="H2" s="89"/>
-      <c r="I2" s="89"/>
-      <c r="J2" s="89"/>
-      <c r="K2" s="90"/>
+      <c r="G2" s="94"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="95"/>
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1711,7 +1714,7 @@
       <c r="A4" s="11">
         <v>1</v>
       </c>
-      <c r="B4" s="91" t="s">
+      <c r="B4" s="96" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="14" t="s">
@@ -1737,7 +1740,7 @@
       <c r="A5" s="11">
         <v>2</v>
       </c>
-      <c r="B5" s="92"/>
+      <c r="B5" s="97"/>
       <c r="C5" s="18" t="s">
         <v>25</v>
       </c>
@@ -1795,7 +1798,7 @@
       <c r="A7" s="11">
         <v>4</v>
       </c>
-      <c r="B7" s="93" t="s">
+      <c r="B7" s="98" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="18" t="s">
@@ -1827,7 +1830,7 @@
       <c r="A8" s="11">
         <v>5</v>
       </c>
-      <c r="B8" s="93"/>
+      <c r="B8" s="98"/>
       <c r="C8" s="18" t="s">
         <v>30</v>
       </c>
@@ -1855,7 +1858,7 @@
       <c r="A9" s="11">
         <v>6</v>
       </c>
-      <c r="B9" s="93"/>
+      <c r="B9" s="98"/>
       <c r="C9" s="18" t="s">
         <v>31</v>
       </c>
@@ -1883,7 +1886,7 @@
       <c r="A10" s="11">
         <v>7</v>
       </c>
-      <c r="B10" s="93"/>
+      <c r="B10" s="98"/>
       <c r="C10" s="18" t="s">
         <v>32</v>
       </c>
@@ -1917,7 +1920,7 @@
       <c r="A11" s="11">
         <v>8</v>
       </c>
-      <c r="B11" s="94" t="s">
+      <c r="B11" s="99" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="28" t="s">
@@ -1953,7 +1956,7 @@
       <c r="A12" s="11">
         <v>9</v>
       </c>
-      <c r="B12" s="95"/>
+      <c r="B12" s="100"/>
       <c r="C12" s="30" t="s">
         <v>35</v>
       </c>
@@ -1987,7 +1990,7 @@
       <c r="A13" s="11">
         <v>10</v>
       </c>
-      <c r="B13" s="95"/>
+      <c r="B13" s="100"/>
       <c r="C13" s="30" t="s">
         <v>36</v>
       </c>
@@ -2021,7 +2024,7 @@
       <c r="A14" s="11">
         <v>11</v>
       </c>
-      <c r="B14" s="95"/>
+      <c r="B14" s="100"/>
       <c r="C14" s="30" t="s">
         <v>37</v>
       </c>
@@ -2051,7 +2054,7 @@
       <c r="A15" s="11">
         <v>12</v>
       </c>
-      <c r="B15" s="95"/>
+      <c r="B15" s="100"/>
       <c r="C15" s="30" t="s">
         <v>38</v>
       </c>
@@ -2073,7 +2076,7 @@
       <c r="A16" s="11">
         <v>13</v>
       </c>
-      <c r="B16" s="95"/>
+      <c r="B16" s="100"/>
       <c r="C16" s="30" t="s">
         <v>39</v>
       </c>
@@ -2097,7 +2100,7 @@
       <c r="A17" s="11">
         <v>14</v>
       </c>
-      <c r="B17" s="95"/>
+      <c r="B17" s="100"/>
       <c r="C17" s="30" t="s">
         <v>40</v>
       </c>
@@ -2121,7 +2124,7 @@
       <c r="A18" s="11">
         <v>15</v>
       </c>
-      <c r="B18" s="95"/>
+      <c r="B18" s="100"/>
       <c r="C18" s="30" t="s">
         <v>41</v>
       </c>
@@ -2145,7 +2148,7 @@
       <c r="A19" s="11">
         <v>16</v>
       </c>
-      <c r="B19" s="95"/>
+      <c r="B19" s="100"/>
       <c r="C19" s="30" t="s">
         <v>42</v>
       </c>
@@ -2169,7 +2172,7 @@
       <c r="A20" s="11">
         <v>17</v>
       </c>
-      <c r="B20" s="95"/>
+      <c r="B20" s="100"/>
       <c r="C20" s="30" t="s">
         <v>43</v>
       </c>
@@ -2191,7 +2194,7 @@
       <c r="A21" s="11">
         <v>18</v>
       </c>
-      <c r="B21" s="96" t="s">
+      <c r="B21" s="101" t="s">
         <v>44</v>
       </c>
       <c r="C21" s="30" t="s">
@@ -2217,7 +2220,7 @@
       <c r="A22" s="11">
         <v>19</v>
       </c>
-      <c r="B22" s="96"/>
+      <c r="B22" s="101"/>
       <c r="C22" s="30" t="s">
         <v>46</v>
       </c>
@@ -2238,7 +2241,7 @@
       <c r="A23" s="11">
         <v>20</v>
       </c>
-      <c r="B23" s="96"/>
+      <c r="B23" s="101"/>
       <c r="C23" s="28" t="s">
         <v>47</v>
       </c>
@@ -2259,7 +2262,7 @@
       <c r="A24" s="11">
         <v>21</v>
       </c>
-      <c r="B24" s="96"/>
+      <c r="B24" s="101"/>
       <c r="C24" s="28" t="s">
         <v>48</v>
       </c>
@@ -2290,7 +2293,7 @@
       <c r="A25" s="11">
         <v>22</v>
       </c>
-      <c r="B25" s="96"/>
+      <c r="B25" s="101"/>
       <c r="C25" s="30" t="s">
         <v>49</v>
       </c>
@@ -2318,7 +2321,7 @@
       <c r="A26" s="11">
         <v>23</v>
       </c>
-      <c r="B26" s="97" t="s">
+      <c r="B26" s="88" t="s">
         <v>50</v>
       </c>
       <c r="C26" s="44" t="s">
@@ -2350,7 +2353,7 @@
       <c r="A27" s="11">
         <v>24</v>
       </c>
-      <c r="B27" s="97"/>
+      <c r="B27" s="88"/>
       <c r="C27" s="44" t="s">
         <v>52</v>
       </c>
@@ -2380,7 +2383,7 @@
       <c r="A28" s="11">
         <v>25</v>
       </c>
-      <c r="B28" s="97"/>
+      <c r="B28" s="88"/>
       <c r="C28" s="44" t="s">
         <v>53</v>
       </c>
@@ -2408,7 +2411,7 @@
       <c r="A29" s="11">
         <v>26</v>
       </c>
-      <c r="B29" s="97"/>
+      <c r="B29" s="88"/>
       <c r="C29" s="44" t="s">
         <v>54</v>
       </c>
@@ -2436,12 +2439,12 @@
       <c r="A30" s="11">
         <v>27</v>
       </c>
-      <c r="B30" s="97"/>
+      <c r="B30" s="88"/>
       <c r="C30" s="44" t="s">
         <v>55</v>
       </c>
       <c r="D30" s="70" t="s">
-        <v>190</v>
+        <v>257</v>
       </c>
       <c r="E30" s="66" t="s">
         <v>11</v>
@@ -2464,7 +2467,7 @@
       <c r="A31" s="11">
         <v>28</v>
       </c>
-      <c r="B31" s="97"/>
+      <c r="B31" s="88"/>
       <c r="C31" s="44" t="s">
         <v>56</v>
       </c>
@@ -2492,7 +2495,7 @@
       <c r="A32" s="11">
         <v>29</v>
       </c>
-      <c r="B32" s="97"/>
+      <c r="B32" s="88"/>
       <c r="C32" s="44" t="s">
         <v>57</v>
       </c>
@@ -2520,7 +2523,7 @@
       <c r="A33" s="11">
         <v>30</v>
       </c>
-      <c r="B33" s="97"/>
+      <c r="B33" s="88"/>
       <c r="C33" s="44" t="s">
         <v>58</v>
       </c>
@@ -2548,7 +2551,7 @@
       <c r="A34" s="11">
         <v>31</v>
       </c>
-      <c r="B34" s="97"/>
+      <c r="B34" s="88"/>
       <c r="C34" s="44" t="s">
         <v>59</v>
       </c>
@@ -2576,7 +2579,7 @@
       <c r="A35" s="11">
         <v>32</v>
       </c>
-      <c r="B35" s="97"/>
+      <c r="B35" s="88"/>
       <c r="C35" s="44" t="s">
         <v>60</v>
       </c>
@@ -2604,7 +2607,7 @@
       <c r="A36" s="11">
         <v>33</v>
       </c>
-      <c r="B36" s="97"/>
+      <c r="B36" s="88"/>
       <c r="C36" s="44" t="s">
         <v>61</v>
       </c>
@@ -2632,7 +2635,7 @@
       <c r="A37" s="11">
         <v>34</v>
       </c>
-      <c r="B37" s="97"/>
+      <c r="B37" s="88"/>
       <c r="C37" s="44" t="s">
         <v>62</v>
       </c>
@@ -2659,7 +2662,7 @@
       <c r="A38" s="11">
         <v>35</v>
       </c>
-      <c r="B38" s="97"/>
+      <c r="B38" s="88"/>
       <c r="C38" s="44" t="s">
         <v>63</v>
       </c>
@@ -2686,7 +2689,7 @@
       <c r="A39" s="11">
         <v>36</v>
       </c>
-      <c r="B39" s="97"/>
+      <c r="B39" s="88"/>
       <c r="C39" s="44" t="s">
         <v>64</v>
       </c>
@@ -2713,7 +2716,7 @@
       <c r="A40" s="11">
         <v>37</v>
       </c>
-      <c r="B40" s="97"/>
+      <c r="B40" s="88"/>
       <c r="C40" s="44" t="s">
         <v>65</v>
       </c>
@@ -2740,7 +2743,7 @@
       <c r="A41" s="11">
         <v>38</v>
       </c>
-      <c r="B41" s="97"/>
+      <c r="B41" s="88"/>
       <c r="C41" s="44" t="s">
         <v>66</v>
       </c>
@@ -2767,7 +2770,7 @@
       <c r="A42" s="11">
         <v>39</v>
       </c>
-      <c r="B42" s="97"/>
+      <c r="B42" s="88"/>
       <c r="C42" s="44" t="s">
         <v>67</v>
       </c>
@@ -2794,7 +2797,7 @@
       <c r="A43" s="11">
         <v>40</v>
       </c>
-      <c r="B43" s="97"/>
+      <c r="B43" s="88"/>
       <c r="C43" s="44" t="s">
         <v>68</v>
       </c>
@@ -2821,7 +2824,7 @@
       <c r="A44" s="11">
         <v>41</v>
       </c>
-      <c r="B44" s="97"/>
+      <c r="B44" s="88"/>
       <c r="C44" s="44" t="s">
         <v>69</v>
       </c>
@@ -2848,7 +2851,7 @@
       <c r="A45" s="11">
         <v>42</v>
       </c>
-      <c r="B45" s="97"/>
+      <c r="B45" s="88"/>
       <c r="C45" s="44" t="s">
         <v>70</v>
       </c>
@@ -2875,7 +2878,7 @@
       <c r="A46" s="11">
         <v>43</v>
       </c>
-      <c r="B46" s="97"/>
+      <c r="B46" s="88"/>
       <c r="C46" s="44" t="s">
         <v>71</v>
       </c>
@@ -2902,7 +2905,7 @@
       <c r="A47" s="11">
         <v>44</v>
       </c>
-      <c r="B47" s="97"/>
+      <c r="B47" s="88"/>
       <c r="C47" s="44" t="s">
         <v>72</v>
       </c>
@@ -2929,7 +2932,7 @@
       <c r="A48" s="11">
         <v>45</v>
       </c>
-      <c r="B48" s="97"/>
+      <c r="B48" s="88"/>
       <c r="C48" s="44" t="s">
         <v>73</v>
       </c>
@@ -2956,7 +2959,7 @@
       <c r="A49" s="11">
         <v>46</v>
       </c>
-      <c r="B49" s="97"/>
+      <c r="B49" s="88"/>
       <c r="C49" s="44" t="s">
         <v>74</v>
       </c>
@@ -2983,7 +2986,7 @@
       <c r="A50" s="11">
         <v>47</v>
       </c>
-      <c r="B50" s="97"/>
+      <c r="B50" s="88"/>
       <c r="C50" s="28" t="s">
         <v>75</v>
       </c>
@@ -3010,7 +3013,7 @@
       <c r="A51" s="11">
         <v>48</v>
       </c>
-      <c r="B51" s="97"/>
+      <c r="B51" s="88"/>
       <c r="C51" s="28" t="s">
         <v>76</v>
       </c>
@@ -3037,7 +3040,7 @@
       <c r="A52" s="11">
         <v>49</v>
       </c>
-      <c r="B52" s="97"/>
+      <c r="B52" s="88"/>
       <c r="C52" s="28" t="s">
         <v>77</v>
       </c>
@@ -3064,7 +3067,7 @@
       <c r="A53" s="11">
         <v>50</v>
       </c>
-      <c r="B53" s="98" t="s">
+      <c r="B53" s="89" t="s">
         <v>78</v>
       </c>
       <c r="C53" s="18" t="s">
@@ -3093,7 +3096,7 @@
       <c r="A54" s="11">
         <v>51</v>
       </c>
-      <c r="B54" s="98"/>
+      <c r="B54" s="89"/>
       <c r="C54" s="18" t="s">
         <v>80</v>
       </c>
@@ -3108,7 +3111,7 @@
       <c r="A55" s="11">
         <v>52</v>
       </c>
-      <c r="B55" s="98"/>
+      <c r="B55" s="89"/>
       <c r="C55" s="45" t="s">
         <v>81</v>
       </c>
@@ -3123,7 +3126,7 @@
       <c r="A56" s="11">
         <v>53</v>
       </c>
-      <c r="B56" s="98"/>
+      <c r="B56" s="89"/>
       <c r="C56" s="45" t="s">
         <v>82</v>
       </c>
@@ -3138,7 +3141,7 @@
       <c r="A57" s="11">
         <v>54</v>
       </c>
-      <c r="B57" s="98"/>
+      <c r="B57" s="89"/>
       <c r="C57" s="30" t="s">
         <v>83</v>
       </c>
@@ -3153,7 +3156,7 @@
       <c r="A58" s="11">
         <v>55</v>
       </c>
-      <c r="B58" s="98"/>
+      <c r="B58" s="89"/>
       <c r="C58" s="45" t="s">
         <v>84</v>
       </c>
@@ -3168,7 +3171,7 @@
       <c r="A59" s="11">
         <v>56</v>
       </c>
-      <c r="B59" s="98"/>
+      <c r="B59" s="89"/>
       <c r="C59" s="45" t="s">
         <v>85</v>
       </c>
@@ -3183,7 +3186,7 @@
       <c r="A60" s="11">
         <v>57</v>
       </c>
-      <c r="B60" s="98"/>
+      <c r="B60" s="89"/>
       <c r="C60" s="18" t="s">
         <v>86</v>
       </c>
@@ -3198,7 +3201,7 @@
       <c r="A61" s="11">
         <v>58</v>
       </c>
-      <c r="B61" s="99" t="s">
+      <c r="B61" s="90" t="s">
         <v>87</v>
       </c>
       <c r="C61" s="45" t="s">
@@ -3215,7 +3218,7 @@
       <c r="A62" s="11">
         <v>59</v>
       </c>
-      <c r="B62" s="99"/>
+      <c r="B62" s="90"/>
       <c r="C62" s="45" t="s">
         <v>89</v>
       </c>
@@ -3230,7 +3233,7 @@
       <c r="A63" s="11">
         <v>60</v>
       </c>
-      <c r="B63" s="99"/>
+      <c r="B63" s="90"/>
       <c r="C63" s="45" t="s">
         <v>90</v>
       </c>
@@ -3245,7 +3248,7 @@
       <c r="A64" s="11">
         <v>61</v>
       </c>
-      <c r="B64" s="99"/>
+      <c r="B64" s="90"/>
       <c r="C64" s="45" t="s">
         <v>91</v>
       </c>
@@ -3260,7 +3263,7 @@
       <c r="A65" s="11">
         <v>62</v>
       </c>
-      <c r="B65" s="99"/>
+      <c r="B65" s="90"/>
       <c r="C65" s="18" t="s">
         <v>92</v>
       </c>
@@ -3273,7 +3276,7 @@
       <c r="A66" s="11">
         <v>63</v>
       </c>
-      <c r="B66" s="99"/>
+      <c r="B66" s="90"/>
       <c r="C66" s="18" t="s">
         <v>93</v>
       </c>
@@ -3286,7 +3289,7 @@
       <c r="A67" s="11">
         <v>64</v>
       </c>
-      <c r="B67" s="99"/>
+      <c r="B67" s="90"/>
       <c r="C67" s="45" t="s">
         <v>94</v>
       </c>
@@ -3299,7 +3302,7 @@
       <c r="A68" s="11">
         <v>65</v>
       </c>
-      <c r="B68" s="100" t="s">
+      <c r="B68" s="91" t="s">
         <v>95</v>
       </c>
       <c r="C68" s="46" t="s">
@@ -3314,7 +3317,7 @@
       <c r="A69" s="11">
         <v>66</v>
       </c>
-      <c r="B69" s="100"/>
+      <c r="B69" s="91"/>
       <c r="C69" s="46" t="s">
         <v>97</v>
       </c>
@@ -3327,7 +3330,7 @@
       <c r="A70" s="11">
         <v>67</v>
       </c>
-      <c r="B70" s="100"/>
+      <c r="B70" s="91"/>
       <c r="C70" s="46" t="s">
         <v>98</v>
       </c>
@@ -3340,7 +3343,7 @@
       <c r="A71" s="11">
         <v>68</v>
       </c>
-      <c r="B71" s="100"/>
+      <c r="B71" s="91"/>
       <c r="C71" s="46" t="s">
         <v>99</v>
       </c>
@@ -3353,7 +3356,7 @@
       <c r="A72" s="11">
         <v>69</v>
       </c>
-      <c r="B72" s="101"/>
+      <c r="B72" s="92"/>
       <c r="C72" s="47" t="s">
         <v>100</v>
       </c>
@@ -3364,16 +3367,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F2:K2"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="B11:B20"/>
+    <mergeCell ref="B21:B25"/>
     <mergeCell ref="B26:B52"/>
     <mergeCell ref="B53:B60"/>
     <mergeCell ref="B61:B67"/>
     <mergeCell ref="B68:B72"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:K2"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="B11:B20"/>
-    <mergeCell ref="B21:B25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Validator Second Review was added.
</commit_message>
<xml_diff>
--- a/IEF_Home/UploadedFiles/1_F_Inputoutput_TABLE_Sample_Test.xlsx
+++ b/IEF_Home/UploadedFiles/1_F_Inputoutput_TABLE_Sample_Test.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20415"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3A2DD7EF-799F-4810-9470-837AE99DF4D2}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3223AAB6-65C4-4C19-A01B-9AAF31515660}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="9330" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1281,21 +1281,6 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1322,6 +1307,21 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1680,20 +1680,20 @@
       <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="93" t="s">
+      <c r="B2" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="94"/>
-      <c r="D2" s="95"/>
+      <c r="C2" s="89"/>
+      <c r="D2" s="90"/>
       <c r="E2" s="66"/>
-      <c r="F2" s="93" t="s">
+      <c r="F2" s="88" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="94"/>
-      <c r="H2" s="94"/>
-      <c r="I2" s="94"/>
-      <c r="J2" s="94"/>
-      <c r="K2" s="95"/>
+      <c r="G2" s="89"/>
+      <c r="H2" s="89"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
+      <c r="K2" s="90"/>
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1714,7 +1714,7 @@
       <c r="A4" s="11">
         <v>1</v>
       </c>
-      <c r="B4" s="96" t="s">
+      <c r="B4" s="91" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="14" t="s">
@@ -1740,7 +1740,7 @@
       <c r="A5" s="11">
         <v>2</v>
       </c>
-      <c r="B5" s="97"/>
+      <c r="B5" s="92"/>
       <c r="C5" s="18" t="s">
         <v>25</v>
       </c>
@@ -1798,7 +1798,7 @@
       <c r="A7" s="11">
         <v>4</v>
       </c>
-      <c r="B7" s="98" t="s">
+      <c r="B7" s="93" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="18" t="s">
@@ -1830,7 +1830,7 @@
       <c r="A8" s="11">
         <v>5</v>
       </c>
-      <c r="B8" s="98"/>
+      <c r="B8" s="93"/>
       <c r="C8" s="18" t="s">
         <v>30</v>
       </c>
@@ -1858,7 +1858,7 @@
       <c r="A9" s="11">
         <v>6</v>
       </c>
-      <c r="B9" s="98"/>
+      <c r="B9" s="93"/>
       <c r="C9" s="18" t="s">
         <v>31</v>
       </c>
@@ -1886,7 +1886,7 @@
       <c r="A10" s="11">
         <v>7</v>
       </c>
-      <c r="B10" s="98"/>
+      <c r="B10" s="93"/>
       <c r="C10" s="18" t="s">
         <v>32</v>
       </c>
@@ -1920,7 +1920,7 @@
       <c r="A11" s="11">
         <v>8</v>
       </c>
-      <c r="B11" s="99" t="s">
+      <c r="B11" s="94" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="28" t="s">
@@ -1956,7 +1956,7 @@
       <c r="A12" s="11">
         <v>9</v>
       </c>
-      <c r="B12" s="100"/>
+      <c r="B12" s="95"/>
       <c r="C12" s="30" t="s">
         <v>35</v>
       </c>
@@ -1990,7 +1990,7 @@
       <c r="A13" s="11">
         <v>10</v>
       </c>
-      <c r="B13" s="100"/>
+      <c r="B13" s="95"/>
       <c r="C13" s="30" t="s">
         <v>36</v>
       </c>
@@ -2024,7 +2024,7 @@
       <c r="A14" s="11">
         <v>11</v>
       </c>
-      <c r="B14" s="100"/>
+      <c r="B14" s="95"/>
       <c r="C14" s="30" t="s">
         <v>37</v>
       </c>
@@ -2054,7 +2054,7 @@
       <c r="A15" s="11">
         <v>12</v>
       </c>
-      <c r="B15" s="100"/>
+      <c r="B15" s="95"/>
       <c r="C15" s="30" t="s">
         <v>38</v>
       </c>
@@ -2076,7 +2076,7 @@
       <c r="A16" s="11">
         <v>13</v>
       </c>
-      <c r="B16" s="100"/>
+      <c r="B16" s="95"/>
       <c r="C16" s="30" t="s">
         <v>39</v>
       </c>
@@ -2100,7 +2100,7 @@
       <c r="A17" s="11">
         <v>14</v>
       </c>
-      <c r="B17" s="100"/>
+      <c r="B17" s="95"/>
       <c r="C17" s="30" t="s">
         <v>40</v>
       </c>
@@ -2124,7 +2124,7 @@
       <c r="A18" s="11">
         <v>15</v>
       </c>
-      <c r="B18" s="100"/>
+      <c r="B18" s="95"/>
       <c r="C18" s="30" t="s">
         <v>41</v>
       </c>
@@ -2148,7 +2148,7 @@
       <c r="A19" s="11">
         <v>16</v>
       </c>
-      <c r="B19" s="100"/>
+      <c r="B19" s="95"/>
       <c r="C19" s="30" t="s">
         <v>42</v>
       </c>
@@ -2172,7 +2172,7 @@
       <c r="A20" s="11">
         <v>17</v>
       </c>
-      <c r="B20" s="100"/>
+      <c r="B20" s="95"/>
       <c r="C20" s="30" t="s">
         <v>43</v>
       </c>
@@ -2194,7 +2194,7 @@
       <c r="A21" s="11">
         <v>18</v>
       </c>
-      <c r="B21" s="101" t="s">
+      <c r="B21" s="96" t="s">
         <v>44</v>
       </c>
       <c r="C21" s="30" t="s">
@@ -2220,7 +2220,7 @@
       <c r="A22" s="11">
         <v>19</v>
       </c>
-      <c r="B22" s="101"/>
+      <c r="B22" s="96"/>
       <c r="C22" s="30" t="s">
         <v>46</v>
       </c>
@@ -2241,7 +2241,7 @@
       <c r="A23" s="11">
         <v>20</v>
       </c>
-      <c r="B23" s="101"/>
+      <c r="B23" s="96"/>
       <c r="C23" s="28" t="s">
         <v>47</v>
       </c>
@@ -2262,7 +2262,7 @@
       <c r="A24" s="11">
         <v>21</v>
       </c>
-      <c r="B24" s="101"/>
+      <c r="B24" s="96"/>
       <c r="C24" s="28" t="s">
         <v>48</v>
       </c>
@@ -2293,7 +2293,7 @@
       <c r="A25" s="11">
         <v>22</v>
       </c>
-      <c r="B25" s="101"/>
+      <c r="B25" s="96"/>
       <c r="C25" s="30" t="s">
         <v>49</v>
       </c>
@@ -2321,7 +2321,7 @@
       <c r="A26" s="11">
         <v>23</v>
       </c>
-      <c r="B26" s="88" t="s">
+      <c r="B26" s="97" t="s">
         <v>50</v>
       </c>
       <c r="C26" s="44" t="s">
@@ -2353,7 +2353,7 @@
       <c r="A27" s="11">
         <v>24</v>
       </c>
-      <c r="B27" s="88"/>
+      <c r="B27" s="97"/>
       <c r="C27" s="44" t="s">
         <v>52</v>
       </c>
@@ -2383,7 +2383,7 @@
       <c r="A28" s="11">
         <v>25</v>
       </c>
-      <c r="B28" s="88"/>
+      <c r="B28" s="97"/>
       <c r="C28" s="44" t="s">
         <v>53</v>
       </c>
@@ -2411,7 +2411,7 @@
       <c r="A29" s="11">
         <v>26</v>
       </c>
-      <c r="B29" s="88"/>
+      <c r="B29" s="97"/>
       <c r="C29" s="44" t="s">
         <v>54</v>
       </c>
@@ -2439,7 +2439,7 @@
       <c r="A30" s="11">
         <v>27</v>
       </c>
-      <c r="B30" s="88"/>
+      <c r="B30" s="97"/>
       <c r="C30" s="44" t="s">
         <v>55</v>
       </c>
@@ -2467,7 +2467,7 @@
       <c r="A31" s="11">
         <v>28</v>
       </c>
-      <c r="B31" s="88"/>
+      <c r="B31" s="97"/>
       <c r="C31" s="44" t="s">
         <v>56</v>
       </c>
@@ -2495,7 +2495,7 @@
       <c r="A32" s="11">
         <v>29</v>
       </c>
-      <c r="B32" s="88"/>
+      <c r="B32" s="97"/>
       <c r="C32" s="44" t="s">
         <v>57</v>
       </c>
@@ -2523,7 +2523,7 @@
       <c r="A33" s="11">
         <v>30</v>
       </c>
-      <c r="B33" s="88"/>
+      <c r="B33" s="97"/>
       <c r="C33" s="44" t="s">
         <v>58</v>
       </c>
@@ -2551,7 +2551,7 @@
       <c r="A34" s="11">
         <v>31</v>
       </c>
-      <c r="B34" s="88"/>
+      <c r="B34" s="97"/>
       <c r="C34" s="44" t="s">
         <v>59</v>
       </c>
@@ -2579,7 +2579,7 @@
       <c r="A35" s="11">
         <v>32</v>
       </c>
-      <c r="B35" s="88"/>
+      <c r="B35" s="97"/>
       <c r="C35" s="44" t="s">
         <v>60</v>
       </c>
@@ -2607,7 +2607,7 @@
       <c r="A36" s="11">
         <v>33</v>
       </c>
-      <c r="B36" s="88"/>
+      <c r="B36" s="97"/>
       <c r="C36" s="44" t="s">
         <v>61</v>
       </c>
@@ -2635,7 +2635,7 @@
       <c r="A37" s="11">
         <v>34</v>
       </c>
-      <c r="B37" s="88"/>
+      <c r="B37" s="97"/>
       <c r="C37" s="44" t="s">
         <v>62</v>
       </c>
@@ -2662,7 +2662,7 @@
       <c r="A38" s="11">
         <v>35</v>
       </c>
-      <c r="B38" s="88"/>
+      <c r="B38" s="97"/>
       <c r="C38" s="44" t="s">
         <v>63</v>
       </c>
@@ -2689,7 +2689,7 @@
       <c r="A39" s="11">
         <v>36</v>
       </c>
-      <c r="B39" s="88"/>
+      <c r="B39" s="97"/>
       <c r="C39" s="44" t="s">
         <v>64</v>
       </c>
@@ -2716,7 +2716,7 @@
       <c r="A40" s="11">
         <v>37</v>
       </c>
-      <c r="B40" s="88"/>
+      <c r="B40" s="97"/>
       <c r="C40" s="44" t="s">
         <v>65</v>
       </c>
@@ -2743,7 +2743,7 @@
       <c r="A41" s="11">
         <v>38</v>
       </c>
-      <c r="B41" s="88"/>
+      <c r="B41" s="97"/>
       <c r="C41" s="44" t="s">
         <v>66</v>
       </c>
@@ -2770,7 +2770,7 @@
       <c r="A42" s="11">
         <v>39</v>
       </c>
-      <c r="B42" s="88"/>
+      <c r="B42" s="97"/>
       <c r="C42" s="44" t="s">
         <v>67</v>
       </c>
@@ -2797,7 +2797,7 @@
       <c r="A43" s="11">
         <v>40</v>
       </c>
-      <c r="B43" s="88"/>
+      <c r="B43" s="97"/>
       <c r="C43" s="44" t="s">
         <v>68</v>
       </c>
@@ -2824,7 +2824,7 @@
       <c r="A44" s="11">
         <v>41</v>
       </c>
-      <c r="B44" s="88"/>
+      <c r="B44" s="97"/>
       <c r="C44" s="44" t="s">
         <v>69</v>
       </c>
@@ -2851,7 +2851,7 @@
       <c r="A45" s="11">
         <v>42</v>
       </c>
-      <c r="B45" s="88"/>
+      <c r="B45" s="97"/>
       <c r="C45" s="44" t="s">
         <v>70</v>
       </c>
@@ -2878,7 +2878,7 @@
       <c r="A46" s="11">
         <v>43</v>
       </c>
-      <c r="B46" s="88"/>
+      <c r="B46" s="97"/>
       <c r="C46" s="44" t="s">
         <v>71</v>
       </c>
@@ -2905,7 +2905,7 @@
       <c r="A47" s="11">
         <v>44</v>
       </c>
-      <c r="B47" s="88"/>
+      <c r="B47" s="97"/>
       <c r="C47" s="44" t="s">
         <v>72</v>
       </c>
@@ -2932,7 +2932,7 @@
       <c r="A48" s="11">
         <v>45</v>
       </c>
-      <c r="B48" s="88"/>
+      <c r="B48" s="97"/>
       <c r="C48" s="44" t="s">
         <v>73</v>
       </c>
@@ -2959,7 +2959,7 @@
       <c r="A49" s="11">
         <v>46</v>
       </c>
-      <c r="B49" s="88"/>
+      <c r="B49" s="97"/>
       <c r="C49" s="44" t="s">
         <v>74</v>
       </c>
@@ -2986,7 +2986,7 @@
       <c r="A50" s="11">
         <v>47</v>
       </c>
-      <c r="B50" s="88"/>
+      <c r="B50" s="97"/>
       <c r="C50" s="28" t="s">
         <v>75</v>
       </c>
@@ -3013,7 +3013,7 @@
       <c r="A51" s="11">
         <v>48</v>
       </c>
-      <c r="B51" s="88"/>
+      <c r="B51" s="97"/>
       <c r="C51" s="28" t="s">
         <v>76</v>
       </c>
@@ -3040,7 +3040,7 @@
       <c r="A52" s="11">
         <v>49</v>
       </c>
-      <c r="B52" s="88"/>
+      <c r="B52" s="97"/>
       <c r="C52" s="28" t="s">
         <v>77</v>
       </c>
@@ -3067,7 +3067,7 @@
       <c r="A53" s="11">
         <v>50</v>
       </c>
-      <c r="B53" s="89" t="s">
+      <c r="B53" s="98" t="s">
         <v>78</v>
       </c>
       <c r="C53" s="18" t="s">
@@ -3096,7 +3096,7 @@
       <c r="A54" s="11">
         <v>51</v>
       </c>
-      <c r="B54" s="89"/>
+      <c r="B54" s="98"/>
       <c r="C54" s="18" t="s">
         <v>80</v>
       </c>
@@ -3111,7 +3111,7 @@
       <c r="A55" s="11">
         <v>52</v>
       </c>
-      <c r="B55" s="89"/>
+      <c r="B55" s="98"/>
       <c r="C55" s="45" t="s">
         <v>81</v>
       </c>
@@ -3126,7 +3126,7 @@
       <c r="A56" s="11">
         <v>53</v>
       </c>
-      <c r="B56" s="89"/>
+      <c r="B56" s="98"/>
       <c r="C56" s="45" t="s">
         <v>82</v>
       </c>
@@ -3141,7 +3141,7 @@
       <c r="A57" s="11">
         <v>54</v>
       </c>
-      <c r="B57" s="89"/>
+      <c r="B57" s="98"/>
       <c r="C57" s="30" t="s">
         <v>83</v>
       </c>
@@ -3156,7 +3156,7 @@
       <c r="A58" s="11">
         <v>55</v>
       </c>
-      <c r="B58" s="89"/>
+      <c r="B58" s="98"/>
       <c r="C58" s="45" t="s">
         <v>84</v>
       </c>
@@ -3171,7 +3171,7 @@
       <c r="A59" s="11">
         <v>56</v>
       </c>
-      <c r="B59" s="89"/>
+      <c r="B59" s="98"/>
       <c r="C59" s="45" t="s">
         <v>85</v>
       </c>
@@ -3186,7 +3186,7 @@
       <c r="A60" s="11">
         <v>57</v>
       </c>
-      <c r="B60" s="89"/>
+      <c r="B60" s="98"/>
       <c r="C60" s="18" t="s">
         <v>86</v>
       </c>
@@ -3201,7 +3201,7 @@
       <c r="A61" s="11">
         <v>58</v>
       </c>
-      <c r="B61" s="90" t="s">
+      <c r="B61" s="99" t="s">
         <v>87</v>
       </c>
       <c r="C61" s="45" t="s">
@@ -3218,7 +3218,7 @@
       <c r="A62" s="11">
         <v>59</v>
       </c>
-      <c r="B62" s="90"/>
+      <c r="B62" s="99"/>
       <c r="C62" s="45" t="s">
         <v>89</v>
       </c>
@@ -3233,7 +3233,7 @@
       <c r="A63" s="11">
         <v>60</v>
       </c>
-      <c r="B63" s="90"/>
+      <c r="B63" s="99"/>
       <c r="C63" s="45" t="s">
         <v>90</v>
       </c>
@@ -3248,7 +3248,7 @@
       <c r="A64" s="11">
         <v>61</v>
       </c>
-      <c r="B64" s="90"/>
+      <c r="B64" s="99"/>
       <c r="C64" s="45" t="s">
         <v>91</v>
       </c>
@@ -3263,7 +3263,7 @@
       <c r="A65" s="11">
         <v>62</v>
       </c>
-      <c r="B65" s="90"/>
+      <c r="B65" s="99"/>
       <c r="C65" s="18" t="s">
         <v>92</v>
       </c>
@@ -3276,7 +3276,7 @@
       <c r="A66" s="11">
         <v>63</v>
       </c>
-      <c r="B66" s="90"/>
+      <c r="B66" s="99"/>
       <c r="C66" s="18" t="s">
         <v>93</v>
       </c>
@@ -3289,7 +3289,7 @@
       <c r="A67" s="11">
         <v>64</v>
       </c>
-      <c r="B67" s="90"/>
+      <c r="B67" s="99"/>
       <c r="C67" s="45" t="s">
         <v>94</v>
       </c>
@@ -3302,7 +3302,7 @@
       <c r="A68" s="11">
         <v>65</v>
       </c>
-      <c r="B68" s="91" t="s">
+      <c r="B68" s="100" t="s">
         <v>95</v>
       </c>
       <c r="C68" s="46" t="s">
@@ -3317,7 +3317,7 @@
       <c r="A69" s="11">
         <v>66</v>
       </c>
-      <c r="B69" s="91"/>
+      <c r="B69" s="100"/>
       <c r="C69" s="46" t="s">
         <v>97</v>
       </c>
@@ -3330,7 +3330,7 @@
       <c r="A70" s="11">
         <v>67</v>
       </c>
-      <c r="B70" s="91"/>
+      <c r="B70" s="100"/>
       <c r="C70" s="46" t="s">
         <v>98</v>
       </c>
@@ -3343,7 +3343,7 @@
       <c r="A71" s="11">
         <v>68</v>
       </c>
-      <c r="B71" s="91"/>
+      <c r="B71" s="100"/>
       <c r="C71" s="46" t="s">
         <v>99</v>
       </c>
@@ -3356,7 +3356,7 @@
       <c r="A72" s="11">
         <v>69</v>
       </c>
-      <c r="B72" s="92"/>
+      <c r="B72" s="101"/>
       <c r="C72" s="47" t="s">
         <v>100</v>
       </c>
@@ -3367,16 +3367,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B26:B52"/>
+    <mergeCell ref="B53:B60"/>
+    <mergeCell ref="B61:B67"/>
+    <mergeCell ref="B68:B72"/>
+    <mergeCell ref="B2:D2"/>
     <mergeCell ref="F2:K2"/>
     <mergeCell ref="B4:B5"/>
     <mergeCell ref="B7:B10"/>
     <mergeCell ref="B11:B20"/>
     <mergeCell ref="B21:B25"/>
-    <mergeCell ref="B26:B52"/>
-    <mergeCell ref="B53:B60"/>
-    <mergeCell ref="B61:B67"/>
-    <mergeCell ref="B68:B72"/>
-    <mergeCell ref="B2:D2"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
Complete Cover sheet + Data Sheet Header Check
</commit_message>
<xml_diff>
--- a/IEF_Home/UploadedFiles/1_F_Inputoutput_TABLE_Sample_Test.xlsx
+++ b/IEF_Home/UploadedFiles/1_F_Inputoutput_TABLE_Sample_Test.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="20415"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3223AAB6-65C4-4C19-A01B-9AAF31515660}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B161444-DA38-4DA3-B6C7-B51890F7F842}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="9330" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1477" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1476" uniqueCount="258">
   <si>
     <t>Format_Version</t>
   </si>
@@ -1281,6 +1281,21 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1307,21 +1322,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="9" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="10" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1680,20 +1680,20 @@
       <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:12" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B2" s="88" t="s">
+      <c r="B2" s="93" t="s">
         <v>18</v>
       </c>
-      <c r="C2" s="89"/>
-      <c r="D2" s="90"/>
+      <c r="C2" s="94"/>
+      <c r="D2" s="95"/>
       <c r="E2" s="66"/>
-      <c r="F2" s="88" t="s">
+      <c r="F2" s="93" t="s">
         <v>19</v>
       </c>
-      <c r="G2" s="89"/>
-      <c r="H2" s="89"/>
-      <c r="I2" s="89"/>
-      <c r="J2" s="89"/>
-      <c r="K2" s="90"/>
+      <c r="G2" s="94"/>
+      <c r="H2" s="94"/>
+      <c r="I2" s="94"/>
+      <c r="J2" s="94"/>
+      <c r="K2" s="95"/>
       <c r="L2" s="1"/>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1714,7 +1714,7 @@
       <c r="A4" s="11">
         <v>1</v>
       </c>
-      <c r="B4" s="91" t="s">
+      <c r="B4" s="96" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="14" t="s">
@@ -1740,7 +1740,7 @@
       <c r="A5" s="11">
         <v>2</v>
       </c>
-      <c r="B5" s="92"/>
+      <c r="B5" s="97"/>
       <c r="C5" s="18" t="s">
         <v>25</v>
       </c>
@@ -1798,7 +1798,7 @@
       <c r="A7" s="11">
         <v>4</v>
       </c>
-      <c r="B7" s="93" t="s">
+      <c r="B7" s="98" t="s">
         <v>28</v>
       </c>
       <c r="C7" s="18" t="s">
@@ -1830,7 +1830,7 @@
       <c r="A8" s="11">
         <v>5</v>
       </c>
-      <c r="B8" s="93"/>
+      <c r="B8" s="98"/>
       <c r="C8" s="18" t="s">
         <v>30</v>
       </c>
@@ -1858,7 +1858,7 @@
       <c r="A9" s="11">
         <v>6</v>
       </c>
-      <c r="B9" s="93"/>
+      <c r="B9" s="98"/>
       <c r="C9" s="18" t="s">
         <v>31</v>
       </c>
@@ -1886,7 +1886,7 @@
       <c r="A10" s="11">
         <v>7</v>
       </c>
-      <c r="B10" s="93"/>
+      <c r="B10" s="98"/>
       <c r="C10" s="18" t="s">
         <v>32</v>
       </c>
@@ -1920,7 +1920,7 @@
       <c r="A11" s="11">
         <v>8</v>
       </c>
-      <c r="B11" s="94" t="s">
+      <c r="B11" s="99" t="s">
         <v>33</v>
       </c>
       <c r="C11" s="28" t="s">
@@ -1956,7 +1956,7 @@
       <c r="A12" s="11">
         <v>9</v>
       </c>
-      <c r="B12" s="95"/>
+      <c r="B12" s="100"/>
       <c r="C12" s="30" t="s">
         <v>35</v>
       </c>
@@ -1990,7 +1990,7 @@
       <c r="A13" s="11">
         <v>10</v>
       </c>
-      <c r="B13" s="95"/>
+      <c r="B13" s="100"/>
       <c r="C13" s="30" t="s">
         <v>36</v>
       </c>
@@ -2024,7 +2024,7 @@
       <c r="A14" s="11">
         <v>11</v>
       </c>
-      <c r="B14" s="95"/>
+      <c r="B14" s="100"/>
       <c r="C14" s="30" t="s">
         <v>37</v>
       </c>
@@ -2054,7 +2054,7 @@
       <c r="A15" s="11">
         <v>12</v>
       </c>
-      <c r="B15" s="95"/>
+      <c r="B15" s="100"/>
       <c r="C15" s="30" t="s">
         <v>38</v>
       </c>
@@ -2076,7 +2076,7 @@
       <c r="A16" s="11">
         <v>13</v>
       </c>
-      <c r="B16" s="95"/>
+      <c r="B16" s="100"/>
       <c r="C16" s="30" t="s">
         <v>39</v>
       </c>
@@ -2100,7 +2100,7 @@
       <c r="A17" s="11">
         <v>14</v>
       </c>
-      <c r="B17" s="95"/>
+      <c r="B17" s="100"/>
       <c r="C17" s="30" t="s">
         <v>40</v>
       </c>
@@ -2124,7 +2124,7 @@
       <c r="A18" s="11">
         <v>15</v>
       </c>
-      <c r="B18" s="95"/>
+      <c r="B18" s="100"/>
       <c r="C18" s="30" t="s">
         <v>41</v>
       </c>
@@ -2148,7 +2148,7 @@
       <c r="A19" s="11">
         <v>16</v>
       </c>
-      <c r="B19" s="95"/>
+      <c r="B19" s="100"/>
       <c r="C19" s="30" t="s">
         <v>42</v>
       </c>
@@ -2172,7 +2172,7 @@
       <c r="A20" s="11">
         <v>17</v>
       </c>
-      <c r="B20" s="95"/>
+      <c r="B20" s="100"/>
       <c r="C20" s="30" t="s">
         <v>43</v>
       </c>
@@ -2194,7 +2194,7 @@
       <c r="A21" s="11">
         <v>18</v>
       </c>
-      <c r="B21" s="96" t="s">
+      <c r="B21" s="101" t="s">
         <v>44</v>
       </c>
       <c r="C21" s="30" t="s">
@@ -2220,7 +2220,7 @@
       <c r="A22" s="11">
         <v>19</v>
       </c>
-      <c r="B22" s="96"/>
+      <c r="B22" s="101"/>
       <c r="C22" s="30" t="s">
         <v>46</v>
       </c>
@@ -2241,7 +2241,7 @@
       <c r="A23" s="11">
         <v>20</v>
       </c>
-      <c r="B23" s="96"/>
+      <c r="B23" s="101"/>
       <c r="C23" s="28" t="s">
         <v>47</v>
       </c>
@@ -2262,7 +2262,7 @@
       <c r="A24" s="11">
         <v>21</v>
       </c>
-      <c r="B24" s="96"/>
+      <c r="B24" s="101"/>
       <c r="C24" s="28" t="s">
         <v>48</v>
       </c>
@@ -2293,7 +2293,7 @@
       <c r="A25" s="11">
         <v>22</v>
       </c>
-      <c r="B25" s="96"/>
+      <c r="B25" s="101"/>
       <c r="C25" s="30" t="s">
         <v>49</v>
       </c>
@@ -2321,7 +2321,7 @@
       <c r="A26" s="11">
         <v>23</v>
       </c>
-      <c r="B26" s="97" t="s">
+      <c r="B26" s="88" t="s">
         <v>50</v>
       </c>
       <c r="C26" s="44" t="s">
@@ -2353,7 +2353,7 @@
       <c r="A27" s="11">
         <v>24</v>
       </c>
-      <c r="B27" s="97"/>
+      <c r="B27" s="88"/>
       <c r="C27" s="44" t="s">
         <v>52</v>
       </c>
@@ -2383,7 +2383,7 @@
       <c r="A28" s="11">
         <v>25</v>
       </c>
-      <c r="B28" s="97"/>
+      <c r="B28" s="88"/>
       <c r="C28" s="44" t="s">
         <v>53</v>
       </c>
@@ -2411,7 +2411,7 @@
       <c r="A29" s="11">
         <v>26</v>
       </c>
-      <c r="B29" s="97"/>
+      <c r="B29" s="88"/>
       <c r="C29" s="44" t="s">
         <v>54</v>
       </c>
@@ -2439,7 +2439,7 @@
       <c r="A30" s="11">
         <v>27</v>
       </c>
-      <c r="B30" s="97"/>
+      <c r="B30" s="88"/>
       <c r="C30" s="44" t="s">
         <v>55</v>
       </c>
@@ -2467,7 +2467,7 @@
       <c r="A31" s="11">
         <v>28</v>
       </c>
-      <c r="B31" s="97"/>
+      <c r="B31" s="88"/>
       <c r="C31" s="44" t="s">
         <v>56</v>
       </c>
@@ -2495,13 +2495,11 @@
       <c r="A32" s="11">
         <v>29</v>
       </c>
-      <c r="B32" s="97"/>
+      <c r="B32" s="88"/>
       <c r="C32" s="44" t="s">
         <v>57</v>
       </c>
-      <c r="D32" s="79" t="s">
-        <v>15</v>
-      </c>
+      <c r="D32" s="79"/>
       <c r="E32" s="66" t="s">
         <v>11</v>
       </c>
@@ -2523,7 +2521,7 @@
       <c r="A33" s="11">
         <v>30</v>
       </c>
-      <c r="B33" s="97"/>
+      <c r="B33" s="88"/>
       <c r="C33" s="44" t="s">
         <v>58</v>
       </c>
@@ -2551,7 +2549,7 @@
       <c r="A34" s="11">
         <v>31</v>
       </c>
-      <c r="B34" s="97"/>
+      <c r="B34" s="88"/>
       <c r="C34" s="44" t="s">
         <v>59</v>
       </c>
@@ -2579,7 +2577,7 @@
       <c r="A35" s="11">
         <v>32</v>
       </c>
-      <c r="B35" s="97"/>
+      <c r="B35" s="88"/>
       <c r="C35" s="44" t="s">
         <v>60</v>
       </c>
@@ -2607,7 +2605,7 @@
       <c r="A36" s="11">
         <v>33</v>
       </c>
-      <c r="B36" s="97"/>
+      <c r="B36" s="88"/>
       <c r="C36" s="44" t="s">
         <v>61</v>
       </c>
@@ -2635,7 +2633,7 @@
       <c r="A37" s="11">
         <v>34</v>
       </c>
-      <c r="B37" s="97"/>
+      <c r="B37" s="88"/>
       <c r="C37" s="44" t="s">
         <v>62</v>
       </c>
@@ -2662,7 +2660,7 @@
       <c r="A38" s="11">
         <v>35</v>
       </c>
-      <c r="B38" s="97"/>
+      <c r="B38" s="88"/>
       <c r="C38" s="44" t="s">
         <v>63</v>
       </c>
@@ -2689,7 +2687,7 @@
       <c r="A39" s="11">
         <v>36</v>
       </c>
-      <c r="B39" s="97"/>
+      <c r="B39" s="88"/>
       <c r="C39" s="44" t="s">
         <v>64</v>
       </c>
@@ -2716,7 +2714,7 @@
       <c r="A40" s="11">
         <v>37</v>
       </c>
-      <c r="B40" s="97"/>
+      <c r="B40" s="88"/>
       <c r="C40" s="44" t="s">
         <v>65</v>
       </c>
@@ -2743,7 +2741,7 @@
       <c r="A41" s="11">
         <v>38</v>
       </c>
-      <c r="B41" s="97"/>
+      <c r="B41" s="88"/>
       <c r="C41" s="44" t="s">
         <v>66</v>
       </c>
@@ -2770,7 +2768,7 @@
       <c r="A42" s="11">
         <v>39</v>
       </c>
-      <c r="B42" s="97"/>
+      <c r="B42" s="88"/>
       <c r="C42" s="44" t="s">
         <v>67</v>
       </c>
@@ -2797,7 +2795,7 @@
       <c r="A43" s="11">
         <v>40</v>
       </c>
-      <c r="B43" s="97"/>
+      <c r="B43" s="88"/>
       <c r="C43" s="44" t="s">
         <v>68</v>
       </c>
@@ -2824,7 +2822,7 @@
       <c r="A44" s="11">
         <v>41</v>
       </c>
-      <c r="B44" s="97"/>
+      <c r="B44" s="88"/>
       <c r="C44" s="44" t="s">
         <v>69</v>
       </c>
@@ -2851,7 +2849,7 @@
       <c r="A45" s="11">
         <v>42</v>
       </c>
-      <c r="B45" s="97"/>
+      <c r="B45" s="88"/>
       <c r="C45" s="44" t="s">
         <v>70</v>
       </c>
@@ -2878,7 +2876,7 @@
       <c r="A46" s="11">
         <v>43</v>
       </c>
-      <c r="B46" s="97"/>
+      <c r="B46" s="88"/>
       <c r="C46" s="44" t="s">
         <v>71</v>
       </c>
@@ -2905,7 +2903,7 @@
       <c r="A47" s="11">
         <v>44</v>
       </c>
-      <c r="B47" s="97"/>
+      <c r="B47" s="88"/>
       <c r="C47" s="44" t="s">
         <v>72</v>
       </c>
@@ -2932,7 +2930,7 @@
       <c r="A48" s="11">
         <v>45</v>
       </c>
-      <c r="B48" s="97"/>
+      <c r="B48" s="88"/>
       <c r="C48" s="44" t="s">
         <v>73</v>
       </c>
@@ -2959,7 +2957,7 @@
       <c r="A49" s="11">
         <v>46</v>
       </c>
-      <c r="B49" s="97"/>
+      <c r="B49" s="88"/>
       <c r="C49" s="44" t="s">
         <v>74</v>
       </c>
@@ -2986,7 +2984,7 @@
       <c r="A50" s="11">
         <v>47</v>
       </c>
-      <c r="B50" s="97"/>
+      <c r="B50" s="88"/>
       <c r="C50" s="28" t="s">
         <v>75</v>
       </c>
@@ -3013,7 +3011,7 @@
       <c r="A51" s="11">
         <v>48</v>
       </c>
-      <c r="B51" s="97"/>
+      <c r="B51" s="88"/>
       <c r="C51" s="28" t="s">
         <v>76</v>
       </c>
@@ -3040,7 +3038,7 @@
       <c r="A52" s="11">
         <v>49</v>
       </c>
-      <c r="B52" s="97"/>
+      <c r="B52" s="88"/>
       <c r="C52" s="28" t="s">
         <v>77</v>
       </c>
@@ -3067,7 +3065,7 @@
       <c r="A53" s="11">
         <v>50</v>
       </c>
-      <c r="B53" s="98" t="s">
+      <c r="B53" s="89" t="s">
         <v>78</v>
       </c>
       <c r="C53" s="18" t="s">
@@ -3096,7 +3094,7 @@
       <c r="A54" s="11">
         <v>51</v>
       </c>
-      <c r="B54" s="98"/>
+      <c r="B54" s="89"/>
       <c r="C54" s="18" t="s">
         <v>80</v>
       </c>
@@ -3111,7 +3109,7 @@
       <c r="A55" s="11">
         <v>52</v>
       </c>
-      <c r="B55" s="98"/>
+      <c r="B55" s="89"/>
       <c r="C55" s="45" t="s">
         <v>81</v>
       </c>
@@ -3126,7 +3124,7 @@
       <c r="A56" s="11">
         <v>53</v>
       </c>
-      <c r="B56" s="98"/>
+      <c r="B56" s="89"/>
       <c r="C56" s="45" t="s">
         <v>82</v>
       </c>
@@ -3141,7 +3139,7 @@
       <c r="A57" s="11">
         <v>54</v>
       </c>
-      <c r="B57" s="98"/>
+      <c r="B57" s="89"/>
       <c r="C57" s="30" t="s">
         <v>83</v>
       </c>
@@ -3156,7 +3154,7 @@
       <c r="A58" s="11">
         <v>55</v>
       </c>
-      <c r="B58" s="98"/>
+      <c r="B58" s="89"/>
       <c r="C58" s="45" t="s">
         <v>84</v>
       </c>
@@ -3171,7 +3169,7 @@
       <c r="A59" s="11">
         <v>56</v>
       </c>
-      <c r="B59" s="98"/>
+      <c r="B59" s="89"/>
       <c r="C59" s="45" t="s">
         <v>85</v>
       </c>
@@ -3186,7 +3184,7 @@
       <c r="A60" s="11">
         <v>57</v>
       </c>
-      <c r="B60" s="98"/>
+      <c r="B60" s="89"/>
       <c r="C60" s="18" t="s">
         <v>86</v>
       </c>
@@ -3201,7 +3199,7 @@
       <c r="A61" s="11">
         <v>58</v>
       </c>
-      <c r="B61" s="99" t="s">
+      <c r="B61" s="90" t="s">
         <v>87</v>
       </c>
       <c r="C61" s="45" t="s">
@@ -3218,7 +3216,7 @@
       <c r="A62" s="11">
         <v>59</v>
       </c>
-      <c r="B62" s="99"/>
+      <c r="B62" s="90"/>
       <c r="C62" s="45" t="s">
         <v>89</v>
       </c>
@@ -3233,7 +3231,7 @@
       <c r="A63" s="11">
         <v>60</v>
       </c>
-      <c r="B63" s="99"/>
+      <c r="B63" s="90"/>
       <c r="C63" s="45" t="s">
         <v>90</v>
       </c>
@@ -3248,7 +3246,7 @@
       <c r="A64" s="11">
         <v>61</v>
       </c>
-      <c r="B64" s="99"/>
+      <c r="B64" s="90"/>
       <c r="C64" s="45" t="s">
         <v>91</v>
       </c>
@@ -3263,7 +3261,7 @@
       <c r="A65" s="11">
         <v>62</v>
       </c>
-      <c r="B65" s="99"/>
+      <c r="B65" s="90"/>
       <c r="C65" s="18" t="s">
         <v>92</v>
       </c>
@@ -3276,7 +3274,7 @@
       <c r="A66" s="11">
         <v>63</v>
       </c>
-      <c r="B66" s="99"/>
+      <c r="B66" s="90"/>
       <c r="C66" s="18" t="s">
         <v>93</v>
       </c>
@@ -3289,7 +3287,7 @@
       <c r="A67" s="11">
         <v>64</v>
       </c>
-      <c r="B67" s="99"/>
+      <c r="B67" s="90"/>
       <c r="C67" s="45" t="s">
         <v>94</v>
       </c>
@@ -3302,7 +3300,7 @@
       <c r="A68" s="11">
         <v>65</v>
       </c>
-      <c r="B68" s="100" t="s">
+      <c r="B68" s="91" t="s">
         <v>95</v>
       </c>
       <c r="C68" s="46" t="s">
@@ -3317,7 +3315,7 @@
       <c r="A69" s="11">
         <v>66</v>
       </c>
-      <c r="B69" s="100"/>
+      <c r="B69" s="91"/>
       <c r="C69" s="46" t="s">
         <v>97</v>
       </c>
@@ -3330,7 +3328,7 @@
       <c r="A70" s="11">
         <v>67</v>
       </c>
-      <c r="B70" s="100"/>
+      <c r="B70" s="91"/>
       <c r="C70" s="46" t="s">
         <v>98</v>
       </c>
@@ -3343,7 +3341,7 @@
       <c r="A71" s="11">
         <v>68</v>
       </c>
-      <c r="B71" s="100"/>
+      <c r="B71" s="91"/>
       <c r="C71" s="46" t="s">
         <v>99</v>
       </c>
@@ -3356,7 +3354,7 @@
       <c r="A72" s="11">
         <v>69</v>
       </c>
-      <c r="B72" s="101"/>
+      <c r="B72" s="92"/>
       <c r="C72" s="47" t="s">
         <v>100</v>
       </c>
@@ -3367,16 +3365,16 @@
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="F2:K2"/>
+    <mergeCell ref="B4:B5"/>
+    <mergeCell ref="B7:B10"/>
+    <mergeCell ref="B11:B20"/>
+    <mergeCell ref="B21:B25"/>
     <mergeCell ref="B26:B52"/>
     <mergeCell ref="B53:B60"/>
     <mergeCell ref="B61:B67"/>
     <mergeCell ref="B68:B72"/>
     <mergeCell ref="B2:D2"/>
-    <mergeCell ref="F2:K2"/>
-    <mergeCell ref="B4:B5"/>
-    <mergeCell ref="B7:B10"/>
-    <mergeCell ref="B11:B20"/>
-    <mergeCell ref="B21:B25"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>